<commit_message>
Update upstream LDAP/mail API paths and email payload
Prepend /ldap to upstream paths for LDAP and mail APIs across several routes (admin/ldap/tree, admin/ldap/user, auth/ldap, auth/login, share/[token]/auth) and update lib/mail.ts and scripts/test-mail.ts to use /ldap/api/v1/mail/send. Also change the mail payload field from body_type to is_html. Updated demands-export.xlsx (binary change). These edits align requests with the upstream service's new /ldap namespace and the mail endpoint's expected payload.
</commit_message>
<xml_diff>
--- a/demands-export.xlsx
+++ b/demands-export.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="119">
   <si>
     <t>需求編號</t>
   </si>
@@ -277,90 +277,57 @@
     <t>刘治安</t>
   </si>
   <si>
-    <t>REQ-2026-020</t>
-  </si>
-  <si>
-    <t>IAM 身分識別系統</t>
-  </si>
-  <si>
-    <t>需求確認</t>
+    <t>REQ-2026-025</t>
+  </si>
+  <si>
+    <t>台達 Forecast 業務系統</t>
+  </si>
+  <si>
+    <t>2026/4/22</t>
+  </si>
+  <si>
+    <t>2026/4/9</t>
+  </si>
+  <si>
+    <t>REQ-2026-026</t>
+  </si>
+  <si>
+    <t>田口實驗分析平台</t>
+  </si>
+  <si>
+    <t>李镇</t>
   </si>
   <si>
     <t>2026/7/31</t>
   </si>
   <si>
-    <t>2026/4/2</t>
-  </si>
-  <si>
-    <t>REQ-2026-021</t>
-  </si>
-  <si>
-    <t>製造部日報整合機器人</t>
+    <t>2026/4/13</t>
+  </si>
+  <si>
+    <t>REQ-2026-027</t>
+  </si>
+  <si>
+    <t>供應商評比系統</t>
+  </si>
+  <si>
+    <t>陈巧玲</t>
+  </si>
+  <si>
+    <t>2026/4/14</t>
+  </si>
+  <si>
+    <t>REQ-2026-028</t>
+  </si>
+  <si>
+    <t>BOM 表自動生成</t>
+  </si>
+  <si>
+    <t>李珊珊</t>
   </si>
   <si>
     <t>2026/8/31</t>
   </si>
   <si>
-    <t>REQ-2026-022</t>
-  </si>
-  <si>
-    <t>HR 績效訪談/評比系統</t>
-  </si>
-  <si>
-    <t>REQ-2026-023</t>
-  </si>
-  <si>
-    <t>全球供應鏈戰情室</t>
-  </si>
-  <si>
-    <t>REQ-2026-024</t>
-  </si>
-  <si>
-    <t>線上溝通平台 ( 即時通訊與會議 )</t>
-  </si>
-  <si>
-    <t>REQ-2026-025</t>
-  </si>
-  <si>
-    <t>台達 Forecast 業務系統</t>
-  </si>
-  <si>
-    <t>2026/4/9</t>
-  </si>
-  <si>
-    <t>REQ-2026-026</t>
-  </si>
-  <si>
-    <t>田口實驗分析平台</t>
-  </si>
-  <si>
-    <t>李镇</t>
-  </si>
-  <si>
-    <t>2026/4/13</t>
-  </si>
-  <si>
-    <t>REQ-2026-027</t>
-  </si>
-  <si>
-    <t>供應商評比系統</t>
-  </si>
-  <si>
-    <t>陈巧玲</t>
-  </si>
-  <si>
-    <t>2026/4/14</t>
-  </si>
-  <si>
-    <t>REQ-2026-028</t>
-  </si>
-  <si>
-    <t>BOM 表自動生成</t>
-  </si>
-  <si>
-    <t>李珊珊</t>
-  </si>
-  <si>
     <t>REQ-2026-029</t>
   </si>
   <si>
@@ -400,7 +367,7 @@
     <t>合計</t>
   </si>
   <si>
-    <t>29%</t>
+    <t>43%</t>
   </si>
 </sst>
 </file>
@@ -425,7 +392,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -460,11 +427,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -515,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -553,18 +515,12 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -906,7 +862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1668,551 +1624,331 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" s="8">
+        <v>18</v>
+      </c>
+      <c r="I18" s="8">
+        <v>18</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" s="10">
+        <v>20</v>
+      </c>
+      <c r="I19" s="10">
+        <v>0</v>
+      </c>
+      <c r="J19" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="L19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H20" s="10">
+        <v>10</v>
+      </c>
+      <c r="I20" s="10">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K20" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H21" s="10">
+        <v>15</v>
+      </c>
+      <c r="I21" s="10">
+        <v>0</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H22" s="10">
+        <v>15</v>
+      </c>
+      <c r="I22" s="10">
+        <v>0</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K22" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="14">
-        <v>100</v>
-      </c>
-      <c r="I18" s="14">
+      <c r="D23" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H23" s="10">
+        <v>14</v>
+      </c>
+      <c r="I23" s="10">
         <v>0</v>
       </c>
-      <c r="J18" s="14" t="s">
+      <c r="J23" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="K18" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="L18" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="N18" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="C19" s="13" t="s">
+      <c r="K23" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M23" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" s="14">
-        <v>12</v>
-      </c>
-      <c r="I19" s="14">
-        <v>0</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="L19" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="M19" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="N19" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="14">
-        <v>15</v>
-      </c>
-      <c r="I20" s="14">
-        <v>0</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K20" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="L20" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="M20" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="N20" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H21" s="14">
-        <v>30</v>
-      </c>
-      <c r="I21" s="14">
-        <v>0</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="L21" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="M21" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="N21" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H22" s="14">
-        <v>33</v>
-      </c>
-      <c r="I22" s="14">
-        <v>0</v>
-      </c>
-      <c r="J22" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K22" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="L22" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="M22" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="N22" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="3" t="s">
+      <c r="D24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H23" s="4">
-        <v>18</v>
-      </c>
-      <c r="I23" s="4">
-        <v>14</v>
-      </c>
-      <c r="J23" s="4" t="s">
+      <c r="H24" s="4">
+        <v>10</v>
+      </c>
+      <c r="I24" s="4">
+        <v>8</v>
+      </c>
+      <c r="J24" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="K23" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N23" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H24" s="10">
-        <v>20</v>
-      </c>
-      <c r="I24" s="10">
-        <v>0</v>
-      </c>
-      <c r="J24" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="K24" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="L24" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M24" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N24" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H25" s="10">
-        <v>10</v>
-      </c>
-      <c r="I25" s="10">
-        <v>0</v>
-      </c>
-      <c r="J25" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="L25" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M25" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N25" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G26" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H26" s="10">
-        <v>15</v>
-      </c>
-      <c r="I26" s="10">
-        <v>0</v>
-      </c>
-      <c r="J26" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="K26" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="L26" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M26" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N26" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="K24" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N24" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B27" s="9" t="s">
+    </row>
+    <row r="26" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="16">
+        <v>440</v>
+      </c>
+      <c r="I26" s="16">
+        <v>189</v>
+      </c>
+      <c r="J26" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H27" s="10">
-        <v>15</v>
-      </c>
-      <c r="I27" s="10">
-        <v>0</v>
-      </c>
-      <c r="J27" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="L27" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M27" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N27" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H28" s="10">
-        <v>14</v>
-      </c>
-      <c r="I28" s="10">
-        <v>0</v>
-      </c>
-      <c r="J28" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="K28" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="L28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="M28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N28" s="9" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="H29" s="12">
-        <v>10</v>
-      </c>
-      <c r="I29" s="12">
-        <v>8</v>
-      </c>
-      <c r="J29" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="K29" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="L29" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="M29" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="N29" s="11" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18">
-        <v>630</v>
-      </c>
-      <c r="I31" s="18">
-        <v>185</v>
-      </c>
-      <c r="J31" s="18" t="s">
-        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>